<commit_message>
style: polish mobile layout ergonomics and remove all uppercase text and classes
</commit_message>
<xml_diff>
--- a/100_LEADS_BARBERSHOP_PITCH_PROSPEK.xlsx
+++ b/100_LEADS_BARBERSHOP_PITCH_PROSPEK.xlsx
@@ -49,7 +49,7 @@
     <t>Catatan</t>
   </si>
   <si>
-    <t>CUKUR HADE BARBERSHOP - CIKUTRA</t>
+    <t>Cukur Hade Barbershop - Cikutra</t>
   </si>
   <si>
     <t>Golden Barbershop</t>
@@ -67,13 +67,13 @@
     <t>Captain Barbershop Greenville</t>
   </si>
   <si>
-    <t>CUKUR HADE BARBERSHOP - LENGKONG KECIL</t>
+    <t>Cukur Hade Barbershop - Lengkong Kecil</t>
   </si>
   <si>
     <t>Chief Barbershop - Pondok Indah</t>
   </si>
   <si>
-    <t>Di Bawah Pohon Barber &amp; Shop MENTENG</t>
+    <t>Di Bawah Pohon Barber &amp; Shop Menteng</t>
   </si>
   <si>
     <t>Captain Barbershop Bandung Cihampelas</t>
@@ -82,10 +82,10 @@
     <t>Brocode Barbershop</t>
   </si>
   <si>
-    <t>CUKUR HADE BARBERSHOP - TSM</t>
-  </si>
-  <si>
-    <t>BARCODE BARBERSHOP</t>
+    <t>Cukur Hade Barbershop - Tsm</t>
+  </si>
+  <si>
+    <t>Barcode Barbershop</t>
   </si>
   <si>
     <t>Brocode Jatinangor</t>
@@ -115,16 +115,16 @@
     <t>Captain Barbershop Tebet</t>
   </si>
   <si>
-    <t>CAPTAIN BARBERSHOP SUMMARECON BEKASI</t>
-  </si>
-  <si>
-    <t>Di Bawah Pohon Barber &amp; Shop PURI 1</t>
+    <t>Captain Barbershop Summarecon Bekasi</t>
+  </si>
+  <si>
+    <t>Di Bawah Pohon Barber &amp; Shop Puri 1</t>
   </si>
   <si>
     <t>Captain Barbershop Meruya Ilir</t>
   </si>
   <si>
-    <t>Captain Barbershop Grand wisata</t>
+    <t>Captain Barbershop Grand Wisata</t>
   </si>
   <si>
     <t>Captain Barbershop Condet</t>
@@ -136,19 +136,19 @@
     <t>Captain Barbershop Sumantri</t>
   </si>
   <si>
-    <t>CHIEF BARBERSHOP - PAKUBUWONO</t>
+    <t>Chief Barbershop - Pakubuwono</t>
   </si>
   <si>
     <t>Captain Barbershop Haji Nawi</t>
   </si>
   <si>
-    <t>Di Bawah Pohon Barber &amp; Shop KEMANG</t>
+    <t>Di Bawah Pohon Barber &amp; Shop Kemang</t>
   </si>
   <si>
     <t>Golden Barber Dago Bandung</t>
   </si>
   <si>
-    <t>BarBerBos • Soerya Sumantri</t>
+    <t>Barberbos • Soerya Sumantri</t>
   </si>
   <si>
     <t>Hairnerds Studio Kebayoran</t>
@@ -157,13 +157,13 @@
     <t>Odysen Barbershop Pondok Labu</t>
   </si>
   <si>
-    <t>BarBerBos • Antapani</t>
-  </si>
-  <si>
-    <t>CHIEF BARBERSHOP - SABANG</t>
-  </si>
-  <si>
-    <t>barberfits • Pandawa</t>
+    <t>Barberbos • Antapani</t>
+  </si>
+  <si>
+    <t>Chief Barbershop - Sabang</t>
+  </si>
+  <si>
+    <t>Barberfits • Pandawa</t>
   </si>
   <si>
     <t>Kanaka Barbershop Cimahi</t>
@@ -175,13 +175,13 @@
     <t>The Cut Rumah Barber - Jalan Lombok, Bandung</t>
   </si>
   <si>
-    <t>BarBerBos • Mekar Wangi</t>
+    <t>Barberbos • Mekar Wangi</t>
   </si>
   <si>
     <t>Captain Barbershop Premiere Sutami Bandung</t>
   </si>
   <si>
-    <t>SUMA Barber</t>
+    <t>Suma Barber</t>
   </si>
   <si>
     <t>Hairnerds Studio Bintaro</t>
@@ -190,7 +190,7 @@
     <t>Culture Barbershop</t>
   </si>
   <si>
-    <t>BarBerBos • Summarecon</t>
+    <t>Barberbos • Summarecon</t>
   </si>
   <si>
     <t>Haircoolest Barbershop | Petojo</t>
@@ -202,7 +202,7 @@
     <t>Chief Barbershop - Como Park</t>
   </si>
   <si>
-    <t>BarBerBos • Padjajaran</t>
+    <t>Barberbos • Padjajaran</t>
   </si>
   <si>
     <t>Captain Barbershop Buah Batu</t>
@@ -214,19 +214,19 @@
     <t>Gentology Barbershop</t>
   </si>
   <si>
-    <t>HAIRSTUDIO SALON &amp; BARBER CIPETE</t>
+    <t>Hairstudio Salon &amp; Barber Cipete</t>
   </si>
   <si>
     <t>Tohang's Barber Cawang</t>
   </si>
   <si>
-    <t>BARBERLABS HQ</t>
+    <t>Barberlabs Hq</t>
   </si>
   <si>
     <t>Urban Haircut Studio</t>
   </si>
   <si>
-    <t>BarBerBos • Progo</t>
+    <t>Barberbos • Progo</t>
   </si>
   <si>
     <t>Travourse | Garuda</t>
@@ -238,7 +238,7 @@
     <t>Theboxteam by Barberbox</t>
   </si>
   <si>
-    <t>BarBerBos • Ramdhan</t>
+    <t>Barberbos • Ramdhan</t>
   </si>
   <si>
     <t>Culture Barbershop Arcamanik</t>
@@ -250,22 +250,22 @@
     <t>Captain Barbershop Bintaro</t>
   </si>
   <si>
-    <t>BarBerBos Naripan</t>
+    <t>Barberbos Naripan</t>
   </si>
   <si>
     <t>Barber Day</t>
   </si>
   <si>
-    <t>Hairnerds Studio Bandung (barbershop &amp; salon)</t>
-  </si>
-  <si>
-    <t>HAIRHAUS Bekasi - Barbershop &amp; Salon</t>
+    <t>Hairnerds Studio Bandung (Barbershop &amp; Salon)</t>
+  </si>
+  <si>
+    <t>Hairhaus Bekasi - Barbershop &amp; Salon</t>
   </si>
   <si>
     <t>Moxie Hair Studio 202 (Barbershop)</t>
   </si>
   <si>
-    <t>CAPTAIN BARBERSHOP DUTAMAS</t>
+    <t>Captain Barbershop Dutamas</t>
   </si>
   <si>
     <t>Bow Barbershop Jelambar</t>
@@ -277,7 +277,7 @@
     <t>Moregan Barbershop Meruya Ilir</t>
   </si>
   <si>
-    <t>AD_BARBER TELKOM</t>
+    <t>Ad_barber Telkom</t>
   </si>
   <si>
     <t>Captain Barbershop Sunda Bandung</t>
@@ -292,19 +292,19 @@
     <t>Marco's Chop Shop Barbershop - Grand Indonesia</t>
   </si>
   <si>
-    <t>BarBerBos Karawang</t>
+    <t>Barberbos Karawang</t>
   </si>
   <si>
     <t>Ramo Barbershop Setiabudi</t>
   </si>
   <si>
-    <t>BarberExpress Kemang Barbershop</t>
+    <t>Barberexpress Kemang Barbershop</t>
   </si>
   <si>
     <t>Captain Barbershop Pakubuwono</t>
   </si>
   <si>
-    <t>MASIF Barber House</t>
+    <t>Masif Barber House</t>
   </si>
   <si>
     <t>Captain Barbershop Tanjung Duren</t>
@@ -313,16 +313,16 @@
     <t>Captain Barbershop Depok</t>
   </si>
   <si>
-    <t>Rock n Roll Haircutting &amp; Makeover</t>
-  </si>
-  <si>
-    <t>MANCAVE BARBERSHOP</t>
-  </si>
-  <si>
-    <t>Groomify Barbershop MONOCHROME</t>
-  </si>
-  <si>
-    <t>BarBerBos • Maskumambang</t>
+    <t>Rock N Roll Haircutting &amp; Makeover</t>
+  </si>
+  <si>
+    <t>Mancave Barbershop</t>
+  </si>
+  <si>
+    <t>Groomify Barbershop Monochrome</t>
+  </si>
+  <si>
+    <t>Barberbos • Maskumambang</t>
   </si>
   <si>
     <t>Captain Barbershop Grogol</t>
@@ -331,7 +331,7 @@
     <t>Big Boyz Barbershop Tebet</t>
   </si>
   <si>
-    <t>BarBerBos • KBP (Kota Baru Parahyangan)</t>
+    <t>Barberbos • Kbp (Kota Baru Parahyangan)</t>
   </si>
   <si>
     <t>Westminster Barber &amp; Coffee</t>
@@ -346,7 +346,7 @@
     <t>Ruang Pangkas</t>
   </si>
   <si>
-    <t>BARBERBAR Lebak Bulus</t>
+    <t>Barberbar Lebak Bulus</t>
   </si>
   <si>
     <t>Bandung</t>
@@ -1231,9 +1231,9 @@
     <t>https://barbershop-web-demo.vercel.app/p/barberbar-lebak-bulus</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *CUKUR HADE BARBERSHOP - CIKUTRA*,
-Salam kenal! Saya perhatikan *CUKUR HADE BARBERSHOP - CIKUTRA* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 4,131 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *CUKUR HADE BARBERSHOP - CIKUTRA*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Cukur Hade Barbershop - Cikutra*,
+Salam kenal! Saya perhatikan *Cukur Hade Barbershop - Cikutra* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 4,131 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Cukur Hade Barbershop - Cikutra*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-cikutra
 Keunggulan sistem website ini:
@@ -1243,7 +1243,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.cukur-hade-barbershop-cik.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *CUKUR HADE BARBERSHOP - CIKUTRA*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Cukur Hade Barbershop - Cikutra*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Golden Barbershop*,
@@ -1321,9 +1321,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Greenville*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *CUKUR HADE BARBERSHOP - LENGKONG KECIL*,
-Salam kenal! Saya perhatikan *CUKUR HADE BARBERSHOP - LENGKONG KECIL* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 2,318 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *CUKUR HADE BARBERSHOP - LENGKONG KECIL*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Cukur Hade Barbershop - Lengkong Kecil*,
+Salam kenal! Saya perhatikan *Cukur Hade Barbershop - Lengkong Kecil* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 2,318 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Cukur Hade Barbershop - Lengkong Kecil*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-lengkong-kecil
 Keunggulan sistem website ini:
@@ -1333,7 +1333,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.cukur-hade-barbershop-len.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *CUKUR HADE BARBERSHOP - LENGKONG KECIL*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Cukur Hade Barbershop - Lengkong Kecil*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Chief Barbershop - Pondok Indah*,
@@ -1351,9 +1351,9 @@
 Terima kasih banyak bro, sukses terus untuk *Chief Barbershop - Pondok Indah*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *Di Bawah Pohon Barber &amp; Shop MENTENG*,
-Salam kenal! Saya perhatikan *Di Bawah Pohon Barber &amp; Shop MENTENG* memiliki reputasi yang sangat keren di Google Maps (4.8 ⭐ dari 2,249 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Di Bawah Pohon Barber &amp; Shop MENTENG*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Di Bawah Pohon Barber &amp; Shop Menteng*,
+Salam kenal! Saya perhatikan *Di Bawah Pohon Barber &amp; Shop Menteng* memiliki reputasi yang sangat keren di Google Maps (4.8 ⭐ dari 2,249 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Di Bawah Pohon Barber &amp; Shop Menteng*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-menteng
 Keunggulan sistem website ini:
@@ -1363,7 +1363,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.di-bawah-pohon-barber-sho.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *Di Bawah Pohon Barber &amp; Shop MENTENG*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Di Bawah Pohon Barber &amp; Shop Menteng*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Bandung Cihampelas*,
@@ -1396,9 +1396,9 @@
 Terima kasih banyak bro, sukses terus untuk *Brocode Barbershop*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *CUKUR HADE BARBERSHOP - TSM*,
-Salam kenal! Saya perhatikan *CUKUR HADE BARBERSHOP - TSM* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 2,050 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *CUKUR HADE BARBERSHOP - TSM*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Cukur Hade Barbershop - Tsm*,
+Salam kenal! Saya perhatikan *Cukur Hade Barbershop - Tsm* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 2,050 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Cukur Hade Barbershop - Tsm*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-tsm
 Keunggulan sistem website ini:
@@ -1408,12 +1408,12 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.cukur-hade-barbershop-tsm.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *CUKUR HADE BARBERSHOP - TSM*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>Halo Bro / Tim Manajemen *BARCODE BARBERSHOP*,
-Salam kenal! Saya perhatikan *BARCODE BARBERSHOP* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,860 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BARCODE BARBERSHOP*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+Terima kasih banyak bro, sukses terus untuk *Cukur Hade Barbershop - Tsm*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>Halo Bro / Tim Manajemen *Barcode Barbershop*,
+Salam kenal! Saya perhatikan *Barcode Barbershop* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,860 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barcode Barbershop*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barcode-barbershop
 Keunggulan sistem website ini:
@@ -1423,7 +1423,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barcode-barbershop.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BARCODE BARBERSHOP*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barcode Barbershop*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Brocode Jatinangor*,
@@ -1561,9 +1561,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Tebet*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *CAPTAIN BARBERSHOP SUMMARECON BEKASI*,
-Salam kenal! Saya perhatikan *CAPTAIN BARBERSHOP SUMMARECON BEKASI* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,520 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *CAPTAIN BARBERSHOP SUMMARECON BEKASI*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Captain Barbershop Summarecon Bekasi*,
+Salam kenal! Saya perhatikan *Captain Barbershop Summarecon Bekasi* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,520 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Captain Barbershop Summarecon Bekasi*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/captain-barbershop-summarecon-bekasi
 Keunggulan sistem website ini:
@@ -1573,12 +1573,12 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.captain-barbershop-summar.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *CAPTAIN BARBERSHOP SUMMARECON BEKASI*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>Halo Bro / Tim Manajemen *Di Bawah Pohon Barber &amp; Shop PURI 1*,
-Salam kenal! Saya perhatikan *Di Bawah Pohon Barber &amp; Shop PURI 1* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,507 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Di Bawah Pohon Barber &amp; Shop PURI 1*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Summarecon Bekasi*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>Halo Bro / Tim Manajemen *Di Bawah Pohon Barber &amp; Shop Puri 1*,
+Salam kenal! Saya perhatikan *Di Bawah Pohon Barber &amp; Shop Puri 1* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,507 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Di Bawah Pohon Barber &amp; Shop Puri 1*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-puri-1
 Keunggulan sistem website ini:
@@ -1588,7 +1588,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.di-bawah-pohon-barber-sho.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *Di Bawah Pohon Barber &amp; Shop PURI 1*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Di Bawah Pohon Barber &amp; Shop Puri 1*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Meruya Ilir*,
@@ -1606,9 +1606,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Meruya Ilir*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *Captain Barbershop Grand wisata*,
-Salam kenal! Saya perhatikan *Captain Barbershop Grand wisata* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,482 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Captain Barbershop Grand wisata*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Captain Barbershop Grand Wisata*,
+Salam kenal! Saya perhatikan *Captain Barbershop Grand Wisata* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,482 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Captain Barbershop Grand Wisata*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/captain-barbershop-grand-wisata
 Keunggulan sistem website ini:
@@ -1618,7 +1618,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.captain-barbershop-grand-.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Grand wisata*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Grand Wisata*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Condet*,
@@ -1666,9 +1666,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Sumantri*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *CHIEF BARBERSHOP - PAKUBUWONO*,
-Salam kenal! Saya perhatikan *CHIEF BARBERSHOP - PAKUBUWONO* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 1,354 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *CHIEF BARBERSHOP - PAKUBUWONO*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Chief Barbershop - Pakubuwono*,
+Salam kenal! Saya perhatikan *Chief Barbershop - Pakubuwono* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 1,354 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Chief Barbershop - Pakubuwono*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/chief-barbershop-pakubuwono
 Keunggulan sistem website ini:
@@ -1678,7 +1678,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.chief-barbershop-pakubuwo.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *CHIEF BARBERSHOP - PAKUBUWONO*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Chief Barbershop - Pakubuwono*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Haji Nawi*,
@@ -1696,9 +1696,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Haji Nawi*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *Di Bawah Pohon Barber &amp; Shop KEMANG*,
-Salam kenal! Saya perhatikan *Di Bawah Pohon Barber &amp; Shop KEMANG* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,319 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Di Bawah Pohon Barber &amp; Shop KEMANG*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Di Bawah Pohon Barber &amp; Shop Kemang*,
+Salam kenal! Saya perhatikan *Di Bawah Pohon Barber &amp; Shop Kemang* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,319 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Di Bawah Pohon Barber &amp; Shop Kemang*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-kemang
 Keunggulan sistem website ini:
@@ -1708,7 +1708,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.di-bawah-pohon-barber-sho.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *Di Bawah Pohon Barber &amp; Shop KEMANG*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Di Bawah Pohon Barber &amp; Shop Kemang*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Golden Barber Dago Bandung*,
@@ -1726,9 +1726,9 @@
 Terima kasih banyak bro, sukses terus untuk *Golden Barber Dago Bandung*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • Soerya Sumantri*,
-Salam kenal! Saya perhatikan *BarBerBos • Soerya Sumantri* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 1,298 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • Soerya Sumantri*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos • Soerya Sumantri*,
+Salam kenal! Saya perhatikan *Barberbos • Soerya Sumantri* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 1,298 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Soerya Sumantri*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-soerya-sumantri
 Keunggulan sistem website ini:
@@ -1738,7 +1738,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-soerya-sumantri.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • Soerya Sumantri*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Soerya Sumantri*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Hairnerds Studio Kebayoran*,
@@ -1771,9 +1771,9 @@
 Terima kasih banyak bro, sukses terus untuk *Odysen Barbershop Pondok Labu*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • Antapani*,
-Salam kenal! Saya perhatikan *BarBerBos • Antapani* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,247 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • Antapani*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos • Antapani*,
+Salam kenal! Saya perhatikan *Barberbos • Antapani* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,247 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Antapani*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-antapani
 Keunggulan sistem website ini:
@@ -1783,12 +1783,12 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-antapani.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • Antapani*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>Halo Bro / Tim Manajemen *CHIEF BARBERSHOP - SABANG*,
-Salam kenal! Saya perhatikan *CHIEF BARBERSHOP - SABANG* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,240 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *CHIEF BARBERSHOP - SABANG*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Antapani*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>Halo Bro / Tim Manajemen *Chief Barbershop - Sabang*,
+Salam kenal! Saya perhatikan *Chief Barbershop - Sabang* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,240 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Chief Barbershop - Sabang*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/chief-barbershop-sabang
 Keunggulan sistem website ini:
@@ -1798,12 +1798,12 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.chief-barbershop-sabang.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *CHIEF BARBERSHOP - SABANG*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>Halo Bro / Tim Manajemen *barberfits • Pandawa*,
-Salam kenal! Saya perhatikan *barberfits • Pandawa* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 1,211 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *barberfits • Pandawa*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+Terima kasih banyak bro, sukses terus untuk *Chief Barbershop - Sabang*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>Halo Bro / Tim Manajemen *Barberfits • Pandawa*,
+Salam kenal! Saya perhatikan *Barberfits • Pandawa* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 1,211 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberfits • Pandawa*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberfits-pandawa
 Keunggulan sistem website ini:
@@ -1813,7 +1813,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberfits-pandawa.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *barberfits • Pandawa*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberfits • Pandawa*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Kanaka Barbershop Cimahi*,
@@ -1861,9 +1861,9 @@
 Terima kasih banyak bro, sukses terus untuk *The Cut Rumah Barber - Jalan Lombok, Bandung*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • Mekar Wangi*,
-Salam kenal! Saya perhatikan *BarBerBos • Mekar Wangi* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,194 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • Mekar Wangi*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos • Mekar Wangi*,
+Salam kenal! Saya perhatikan *Barberbos • Mekar Wangi* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,194 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Mekar Wangi*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-mekar-wangi
 Keunggulan sistem website ini:
@@ -1873,7 +1873,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-mekar-wangi.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • Mekar Wangi*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Mekar Wangi*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Premiere Sutami Bandung*,
@@ -1891,9 +1891,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Premiere Sutami Bandung*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *SUMA Barber*,
-Salam kenal! Saya perhatikan *SUMA Barber* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 1,127 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *SUMA Barber*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Suma Barber*,
+Salam kenal! Saya perhatikan *Suma Barber* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 1,127 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Suma Barber*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/suma-barber
 Keunggulan sistem website ini:
@@ -1903,7 +1903,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.suma-barber.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *SUMA Barber*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Suma Barber*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Hairnerds Studio Bintaro*,
@@ -1936,9 +1936,9 @@
 Terima kasih banyak bro, sukses terus untuk *Culture Barbershop*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • Summarecon*,
-Salam kenal! Saya perhatikan *BarBerBos • Summarecon* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,060 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • Summarecon*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos • Summarecon*,
+Salam kenal! Saya perhatikan *Barberbos • Summarecon* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 1,060 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Summarecon*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-summarecon
 Keunggulan sistem website ini:
@@ -1948,7 +1948,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-summarecon.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • Summarecon*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Summarecon*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Haircoolest Barbershop | Petojo*,
@@ -1996,9 +1996,9 @@
 Terima kasih banyak bro, sukses terus untuk *Chief Barbershop - Como Park*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • Padjajaran*,
-Salam kenal! Saya perhatikan *BarBerBos • Padjajaran* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 984 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • Padjajaran*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos • Padjajaran*,
+Salam kenal! Saya perhatikan *Barberbos • Padjajaran* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 984 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Padjajaran*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-padjajaran
 Keunggulan sistem website ini:
@@ -2008,7 +2008,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-padjajaran.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • Padjajaran*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Padjajaran*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Buah Batu*,
@@ -2056,9 +2056,9 @@
 Terima kasih banyak bro, sukses terus untuk *Gentology Barbershop*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *HAIRSTUDIO SALON &amp; BARBER CIPETE*,
-Salam kenal! Saya perhatikan *HAIRSTUDIO SALON &amp; BARBER CIPETE* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 870 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *HAIRSTUDIO SALON &amp; BARBER CIPETE*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Hairstudio Salon &amp; Barber Cipete*,
+Salam kenal! Saya perhatikan *Hairstudio Salon &amp; Barber Cipete* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 870 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Hairstudio Salon &amp; Barber Cipete*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/hairstudio-salon-barber-cipete
 Keunggulan sistem website ini:
@@ -2068,7 +2068,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.hairstudio-salon-barber-c.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *HAIRSTUDIO SALON &amp; BARBER CIPETE*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Hairstudio Salon &amp; Barber Cipete*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Tohang's Barber Cawang*,
@@ -2086,9 +2086,9 @@
 Terima kasih banyak bro, sukses terus untuk *Tohang's Barber Cawang*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BARBERLABS HQ*,
-Salam kenal! Saya perhatikan *BARBERLABS HQ* memiliki reputasi yang sangat keren di Google Maps (4.8 ⭐ dari 845 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BARBERLABS HQ*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberlabs Hq*,
+Salam kenal! Saya perhatikan *Barberlabs Hq* memiliki reputasi yang sangat keren di Google Maps (4.8 ⭐ dari 845 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberlabs Hq*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberlabs-hq
 Keunggulan sistem website ini:
@@ -2098,7 +2098,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberlabs-hq.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BARBERLABS HQ*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberlabs Hq*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Urban Haircut Studio*,
@@ -2116,9 +2116,9 @@
 Terima kasih banyak bro, sukses terus untuk *Urban Haircut Studio*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • Progo*,
-Salam kenal! Saya perhatikan *BarBerBos • Progo* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 797 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • Progo*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos • Progo*,
+Salam kenal! Saya perhatikan *Barberbos • Progo* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 797 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Progo*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-progo
 Keunggulan sistem website ini:
@@ -2128,7 +2128,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-progo.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • Progo*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Progo*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Travourse | Garuda*,
@@ -2176,9 +2176,9 @@
 Terima kasih banyak bro, sukses terus untuk *Theboxteam by Barberbox*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • Ramdhan*,
-Salam kenal! Saya perhatikan *BarBerBos • Ramdhan* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 771 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • Ramdhan*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos • Ramdhan*,
+Salam kenal! Saya perhatikan *Barberbos • Ramdhan* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 771 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Ramdhan*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-ramdhan
 Keunggulan sistem website ini:
@@ -2188,7 +2188,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-ramdhan.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • Ramdhan*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Ramdhan*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Culture Barbershop Arcamanik*,
@@ -2236,9 +2236,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Bintaro*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos Naripan*,
-Salam kenal! Saya perhatikan *BarBerBos Naripan* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 758 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos Naripan*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos Naripan*,
+Salam kenal! Saya perhatikan *Barberbos Naripan* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 758 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos Naripan*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-naripan
 Keunggulan sistem website ini:
@@ -2248,7 +2248,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-naripan.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos Naripan*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos Naripan*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Barber Day*,
@@ -2266,9 +2266,9 @@
 Terima kasih banyak bro, sukses terus untuk *Barber Day*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *Hairnerds Studio Bandung (barbershop &amp; salon)*,
-Salam kenal! Saya perhatikan *Hairnerds Studio Bandung (barbershop &amp; salon)* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 744 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Hairnerds Studio Bandung (barbershop &amp; salon)*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Hairnerds Studio Bandung (Barbershop &amp; Salon)*,
+Salam kenal! Saya perhatikan *Hairnerds Studio Bandung (Barbershop &amp; Salon)* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 744 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Hairnerds Studio Bandung (Barbershop &amp; Salon)*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/hairnerds-studio-bandung-barbershop-salon
 Keunggulan sistem website ini:
@@ -2278,12 +2278,12 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.hairnerds-studio-bandung-.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *Hairnerds Studio Bandung (barbershop &amp; salon)*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>Halo Bro / Tim Manajemen *HAIRHAUS Bekasi - Barbershop &amp; Salon*,
-Salam kenal! Saya perhatikan *HAIRHAUS Bekasi - Barbershop &amp; Salon* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 740 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *HAIRHAUS Bekasi - Barbershop &amp; Salon*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+Terima kasih banyak bro, sukses terus untuk *Hairnerds Studio Bandung (Barbershop &amp; Salon)*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>Halo Bro / Tim Manajemen *Hairhaus Bekasi - Barbershop &amp; Salon*,
+Salam kenal! Saya perhatikan *Hairhaus Bekasi - Barbershop &amp; Salon* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 740 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Hairhaus Bekasi - Barbershop &amp; Salon*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/hairhaus-bekasi-barbershop-salon
 Keunggulan sistem website ini:
@@ -2293,7 +2293,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.hairhaus-bekasi-barbersho.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *HAIRHAUS Bekasi - Barbershop &amp; Salon*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Hairhaus Bekasi - Barbershop &amp; Salon*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Moxie Hair Studio 202 (Barbershop)*,
@@ -2311,9 +2311,9 @@
 Terima kasih banyak bro, sukses terus untuk *Moxie Hair Studio 202 (Barbershop)*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *CAPTAIN BARBERSHOP DUTAMAS*,
-Salam kenal! Saya perhatikan *CAPTAIN BARBERSHOP DUTAMAS* memiliki reputasi yang sangat keren di Google Maps (4.6 ⭐ dari 699 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *CAPTAIN BARBERSHOP DUTAMAS*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Captain Barbershop Dutamas*,
+Salam kenal! Saya perhatikan *Captain Barbershop Dutamas* memiliki reputasi yang sangat keren di Google Maps (4.6 ⭐ dari 699 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Captain Barbershop Dutamas*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/captain-barbershop-dutamas
 Keunggulan sistem website ini:
@@ -2323,7 +2323,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.captain-barbershop-dutama.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *CAPTAIN BARBERSHOP DUTAMAS*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Dutamas*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Bow Barbershop Jelambar*,
@@ -2371,9 +2371,9 @@
 Terima kasih banyak bro, sukses terus untuk *Moregan Barbershop Meruya Ilir*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *AD_BARBER TELKOM*,
-Salam kenal! Saya perhatikan *AD_BARBER TELKOM* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 682 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *AD_BARBER TELKOM*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Ad_barber Telkom*,
+Salam kenal! Saya perhatikan *Ad_barber Telkom* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 682 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Ad_barber Telkom*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/adbarber-telkom
 Keunggulan sistem website ini:
@@ -2383,7 +2383,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.adbarber-telkom.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *AD_BARBER TELKOM*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Ad_barber Telkom*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Sunda Bandung*,
@@ -2446,9 +2446,9 @@
 Terima kasih banyak bro, sukses terus untuk *Marco's Chop Shop Barbershop - Grand Indonesia*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos Karawang*,
-Salam kenal! Saya perhatikan *BarBerBos Karawang* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 657 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos Karawang*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos Karawang*,
+Salam kenal! Saya perhatikan *Barberbos Karawang* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 657 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos Karawang*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-karawang
 Keunggulan sistem website ini:
@@ -2458,7 +2458,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-karawang.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos Karawang*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos Karawang*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Ramo Barbershop Setiabudi*,
@@ -2476,9 +2476,9 @@
 Terima kasih banyak bro, sukses terus untuk *Ramo Barbershop Setiabudi*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarberExpress Kemang Barbershop*,
-Salam kenal! Saya perhatikan *BarberExpress Kemang Barbershop* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 622 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarberExpress Kemang Barbershop*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberexpress Kemang Barbershop*,
+Salam kenal! Saya perhatikan *Barberexpress Kemang Barbershop* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 622 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberexpress Kemang Barbershop*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberexpress-kemang-barbershop
 Keunggulan sistem website ini:
@@ -2488,7 +2488,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberexpress-kemang-barb.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarberExpress Kemang Barbershop*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberexpress Kemang Barbershop*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Pakubuwono*,
@@ -2506,9 +2506,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Pakubuwono*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *MASIF Barber House*,
-Salam kenal! Saya perhatikan *MASIF Barber House* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 619 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *MASIF Barber House*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Masif Barber House*,
+Salam kenal! Saya perhatikan *Masif Barber House* memiliki reputasi yang sangat keren di Google Maps (5.0 ⭐ dari 619 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Masif Barber House*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/masif-barber-house
 Keunggulan sistem website ini:
@@ -2518,7 +2518,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.masif-barber-house.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *MASIF Barber House*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Masif Barber House*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Tanjung Duren*,
@@ -2551,9 +2551,9 @@
 Terima kasih banyak bro, sukses terus untuk *Captain Barbershop Depok*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *Rock n Roll Haircutting &amp; Makeover*,
-Salam kenal! Saya perhatikan *Rock n Roll Haircutting &amp; Makeover* memiliki reputasi yang sangat keren di Google Maps (4.5 ⭐ dari 606 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Rock n Roll Haircutting &amp; Makeover*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Rock N Roll Haircutting &amp; Makeover*,
+Salam kenal! Saya perhatikan *Rock N Roll Haircutting &amp; Makeover* memiliki reputasi yang sangat keren di Google Maps (4.5 ⭐ dari 606 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Rock N Roll Haircutting &amp; Makeover*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/rock-n-roll-haircutting-makeover
 Keunggulan sistem website ini:
@@ -2563,12 +2563,12 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.rock-n-roll-haircutting-m.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *Rock n Roll Haircutting &amp; Makeover*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>Halo Bro / Tim Manajemen *MANCAVE BARBERSHOP*,
-Salam kenal! Saya perhatikan *MANCAVE BARBERSHOP* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 593 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *MANCAVE BARBERSHOP*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+Terima kasih banyak bro, sukses terus untuk *Rock N Roll Haircutting &amp; Makeover*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>Halo Bro / Tim Manajemen *Mancave Barbershop*,
+Salam kenal! Saya perhatikan *Mancave Barbershop* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 593 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Mancave Barbershop*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/mancave-barbershop
 Keunggulan sistem website ini:
@@ -2578,12 +2578,12 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.mancave-barbershop.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *MANCAVE BARBERSHOP*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>Halo Bro / Tim Manajemen *Groomify Barbershop MONOCHROME*,
-Salam kenal! Saya perhatikan *Groomify Barbershop MONOCHROME* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 590 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Groomify Barbershop MONOCHROME*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+Terima kasih banyak bro, sukses terus untuk *Mancave Barbershop*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>Halo Bro / Tim Manajemen *Groomify Barbershop Monochrome*,
+Salam kenal! Saya perhatikan *Groomify Barbershop Monochrome* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 590 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Groomify Barbershop Monochrome*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/groomify-barbershop-monochrome
 Keunggulan sistem website ini:
@@ -2593,12 +2593,12 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.groomify-barbershop-monoc.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *Groomify Barbershop MONOCHROME*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • Maskumambang*,
-Salam kenal! Saya perhatikan *BarBerBos • Maskumambang* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 588 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • Maskumambang*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+Terima kasih banyak bro, sukses terus untuk *Groomify Barbershop Monochrome*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>Halo Bro / Tim Manajemen *Barberbos • Maskumambang*,
+Salam kenal! Saya perhatikan *Barberbos • Maskumambang* memiliki reputasi yang sangat keren di Google Maps (4.9 ⭐ dari 588 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Maskumambang*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-maskumambang
 Keunggulan sistem website ini:
@@ -2608,7 +2608,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-maskumambang.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • Maskumambang*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Maskumambang*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Captain Barbershop Grogol*,
@@ -2641,9 +2641,9 @@
 Terima kasih banyak bro, sukses terus untuk *Big Boyz Barbershop Tebet*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BarBerBos • KBP (Kota Baru Parahyangan)*,
-Salam kenal! Saya perhatikan *BarBerBos • KBP (Kota Baru Parahyangan)* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 577 ulasan pelanggan di Bandung).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BarBerBos • KBP (Kota Baru Parahyangan)*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbos • Kbp (Kota Baru Parahyangan)*,
+Salam kenal! Saya perhatikan *Barberbos • Kbp (Kota Baru Parahyangan)* memiliki reputasi yang sangat keren di Google Maps (4.7 ⭐ dari 577 ulasan pelanggan di Bandung).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbos • Kbp (Kota Baru Parahyangan)*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbos-kbp-kota-baru-parahyangan
 Keunggulan sistem website ini:
@@ -2653,7 +2653,7 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbos-kbp-kota-baru-p.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BarBerBos • KBP (Kota Baru Parahyangan)*! 🙏✂️</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbos • Kbp (Kota Baru Parahyangan)*! 🙏✂️</t>
   </si>
   <si>
     <t>Halo Bro / Tim Manajemen *Westminster Barber &amp; Coffee*,
@@ -2716,9 +2716,9 @@
 Terima kasih banyak bro, sukses terus untuk *Ruang Pangkas*! 🙏✂️</t>
   </si>
   <si>
-    <t>Halo Bro / Tim Manajemen *BARBERBAR Lebak Bulus*,
-Salam kenal! Saya perhatikan *BARBERBAR Lebak Bulus* memiliki reputasi yang sangat keren di Google Maps (4.5 ⭐ dari 555 ulasan pelanggan di Jakarta Selatan).
-Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *BARBERBAR Lebak Bulus*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
+    <t>Halo Bro / Tim Manajemen *Barberbar Lebak Bulus*,
+Salam kenal! Saya perhatikan *Barberbar Lebak Bulus* memiliki reputasi yang sangat keren di Google Maps (4.5 ⭐ dari 555 ulasan pelanggan di Jakarta Selatan).
+Melihat antusiasme pelanggan yang begitu tinggi, kami berinisiatif membuatkan preview website profil modern khusus untuk *Barberbar Lebak Bulus*, lengkap dengan sistem reservasi WhatsApp otomatis langsung ke nomor Anda:
 👉 Akses Website Demo Barbershop Anda di sini:
 https://barbershop-web-demo.vercel.app/p/barberbar-lebak-bulus
 Keunggulan sistem website ini:
@@ -2728,10 +2728,10 @@
 • Hairstyle Lookbook &amp; Face-Shape Guide: Edukasi gaya rambut untuk pelanggan Anda
 • Siap Dihubungkan ke Domain Resmi (contoh: www.barberbar-lebak-bulus.com)
 Website ini sudah siap pakai dan siap kami serahkan. Jika Anda atau tim manajemen tertarik untuk mengaktifkannya, bisa langsung hubungi WhatsApp saya di +62 857-1820-3535 atau klik tombol 'Klaim Website Ini' di halaman demo.
-Terima kasih banyak bro, sukses terus untuk *BARBERBAR Lebak Bulus*! 🙏✂️</t>
-  </si>
-  <si>
-    <t>https://wa.me/6288224362774?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20CIKUTRA%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20CIKUTRA%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%204%2C131%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20CIKUTRA%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-cikutra%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280882-2436-2774%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.cukur-hade-barbershop-cik.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20CIKUTRA%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+Terima kasih banyak bro, sukses terus untuk *Barberbar Lebak Bulus*! 🙏✂️</t>
+  </si>
+  <si>
+    <t>https://wa.me/6288224362774?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACukur%20Hade%20Barbershop%20-%20Cikutra%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACukur%20Hade%20Barbershop%20-%20Cikutra%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%204%2C131%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACukur%20Hade%20Barbershop%20-%20Cikutra%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-cikutra%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280882-2436-2774%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.cukur-hade-barbershop-cik.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACukur%20Hade%20Barbershop%20-%20Cikutra%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281214807192?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AGolden%20Barbershop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AGolden%20Barbershop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%203%2C341%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AGolden%20Barbershop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/golden-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-1480-7192%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.golden-barbershop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AGolden%20Barbershop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2749,13 +2749,13 @@
     <t>https://wa.me/6282142011161?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Greenville%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Greenville%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%202%2C433%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Greenville%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-greenville%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-4201-1161%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-greenv.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Greenville%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6288224362774?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20LENGKONG%20KECIL%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20LENGKONG%20KECIL%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%202%2C318%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20LENGKONG%20KECIL%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-lengkong-kecil%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280882-2436-2774%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.cukur-hade-barbershop-len.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20LENGKONG%20KECIL%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6288224362774?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACukur%20Hade%20Barbershop%20-%20Lengkong%20Kecil%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACukur%20Hade%20Barbershop%20-%20Lengkong%20Kecil%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%202%2C318%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACukur%20Hade%20Barbershop%20-%20Lengkong%20Kecil%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-lengkong-kecil%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280882-2436-2774%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.cukur-hade-barbershop-len.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACukur%20Hade%20Barbershop%20-%20Lengkong%20Kecil%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6287880937999?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AChief%20Barbershop%20-%20Pondok%20Indah%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AChief%20Barbershop%20-%20Pondok%20Indah%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%202%2C292%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AChief%20Barbershop%20-%20Pondok%20Indah%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/chief-barbershop-pondok-indah%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280878-8093-7999%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.chief-barbershop-pondok-i.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AChief%20Barbershop%20-%20Pondok%20Indah%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/628982851456?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20MENTENG%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20MENTENG%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%202%2C249%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20MENTENG%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-menteng%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280898-2851-456%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.di-bawah-pohon-barber-sho.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20MENTENG%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/628982851456?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Menteng%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Menteng%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%202%2C249%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Menteng%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-menteng%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280898-2851-456%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.di-bawah-pohon-barber-sho.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Menteng%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281388088550?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Bandung%20Cihampelas%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Bandung%20Cihampelas%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%202%2C215%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Bandung%20Cihampelas%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-bandung-cihampelas%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280813-8808-8550%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-bandun.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Bandung%20Cihampelas%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2764,10 +2764,10 @@
     <t>https://wa.me/6287792072014?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABrocode%20Barbershop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABrocode%20Barbershop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%202%2C146%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABrocode%20Barbershop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/brocode-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280877-9207-2014%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.brocode-barbershop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABrocode%20Barbershop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6288224362774?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20TSM%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20TSM%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%202%2C050%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20TSM%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-tsm%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280882-2436-2774%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.cukur-hade-barbershop-tsm.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACUKUR%20HADE%20BARBERSHOP%20-%20TSM%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
-  </si>
-  <si>
-    <t>https://wa.me/622122682856?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABARCODE%20BARBERSHOP%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABARCODE%20BARBERSHOP%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C860%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABARCODE%20BARBERSHOP%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barcode-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28021%29%2022682856%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barcode-barbershop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABARCODE%20BARBERSHOP%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6288224362774?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACukur%20Hade%20Barbershop%20-%20Tsm%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACukur%20Hade%20Barbershop%20-%20Tsm%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%202%2C050%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACukur%20Hade%20Barbershop%20-%20Tsm%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/cukur-hade-barbershop-tsm%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280882-2436-2774%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.cukur-hade-barbershop-tsm.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACukur%20Hade%20Barbershop%20-%20Tsm%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+  </si>
+  <si>
+    <t>https://wa.me/622122682856?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarcode%20Barbershop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarcode%20Barbershop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C860%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarcode%20Barbershop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barcode-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28021%29%2022682856%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barcode-barbershop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarcode%20Barbershop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/622287703846?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABrocode%20Jatinangor%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABrocode%20Jatinangor%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C829%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABrocode%20Jatinangor%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/brocode-jatinangor%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28022%29%2087703846%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.brocode-jatinangor.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABrocode%20Jatinangor%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2797,16 +2797,16 @@
     <t>https://wa.me/6282338195903?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Tebet%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Tebet%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%201%2C690%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Tebet%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-tebet%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280823-3819-5903%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-tebet.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Tebet%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6282142011182?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACAPTAIN%20BARBERSHOP%20SUMMARECON%20BEKASI%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACAPTAIN%20BARBERSHOP%20SUMMARECON%20BEKASI%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C520%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACAPTAIN%20BARBERSHOP%20SUMMARECON%20BEKASI%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-summarecon-bekasi%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-4201-1182%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-summar.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACAPTAIN%20BARBERSHOP%20SUMMARECON%20BEKASI%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
-  </si>
-  <si>
-    <t>https://wa.me/628111988327?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20PURI%201%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20PURI%201%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C507%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20PURI%201%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-puri-1%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280811-1988-327%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.di-bawah-pohon-barber-sho.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20PURI%201%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6282142011182?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Summarecon%20Bekasi%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Summarecon%20Bekasi%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C520%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Summarecon%20Bekasi%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-summarecon-bekasi%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-4201-1182%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-summar.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Summarecon%20Bekasi%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+  </si>
+  <si>
+    <t>https://wa.me/628111988327?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Puri%201%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Puri%201%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C507%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Puri%201%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-puri-1%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280811-1988-327%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.di-bawah-pohon-barber-sho.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Puri%201%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281382540002?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Meruya%20Ilir%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Meruya%20Ilir%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%201%2C494%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Meruya%20Ilir%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-meruya-ilir%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280813-8254-0002%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-meruya.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Meruya%20Ilir%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6282142011183?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Grand%20wisata%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Grand%20wisata%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C482%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Grand%20wisata%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-grand-wisata%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-4201-1183%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-grand-.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Grand%20wisata%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6282142011183?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Grand%20Wisata%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Grand%20Wisata%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C482%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Grand%20Wisata%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-grand-wisata%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-4201-1183%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-grand-.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Grand%20Wisata%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6285211265631?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Condet%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Condet%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%201%2C452%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Condet%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-condet%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280852-1126-5631%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-condet.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Condet%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2818,19 +2818,19 @@
     <t>https://wa.me/6285353306743?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Sumantri%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Sumantri%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C371%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Sumantri%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-sumantri%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280853-5330-6743%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-sumant.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Sumantri%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/628172321088?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACHIEF%20BARBERSHOP%20-%20PAKUBUWONO%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACHIEF%20BARBERSHOP%20-%20PAKUBUWONO%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%201%2C354%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACHIEF%20BARBERSHOP%20-%20PAKUBUWONO%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/chief-barbershop-pakubuwono%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280817-2321-088%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.chief-barbershop-pakubuwo.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACHIEF%20BARBERSHOP%20-%20PAKUBUWONO%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/628172321088?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AChief%20Barbershop%20-%20Pakubuwono%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AChief%20Barbershop%20-%20Pakubuwono%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%201%2C354%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AChief%20Barbershop%20-%20Pakubuwono%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/chief-barbershop-pakubuwono%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280817-2321-088%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.chief-barbershop-pakubuwo.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AChief%20Barbershop%20-%20Pakubuwono%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6282121255893?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Haji%20Nawi%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Haji%20Nawi%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%201%2C320%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Haji%20Nawi%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-haji-nawi%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-2125-5893%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-haji-n.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Haji%20Nawi%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6285947410623?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20KEMANG%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20KEMANG%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C319%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20KEMANG%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-kemang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280859-4741-0623%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.di-bawah-pohon-barber-sho.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20KEMANG%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6285947410623?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Kemang%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Kemang%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C319%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Kemang%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/di-bawah-pohon-barber-shop-kemang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280859-4741-0623%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.di-bawah-pohon-barber-sho.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ADi%20Bawah%20Pohon%20Barber%20%26%20Shop%20Kemang%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281214807192?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AGolden%20Barber%20Dago%20Bandung%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AGolden%20Barber%20Dago%20Bandung%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%201%2C313%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AGolden%20Barber%20Dago%20Bandung%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/golden-barber-dago-bandung%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-1480-7192%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.golden-barber-dago-bandun.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AGolden%20Barber%20Dago%20Bandung%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/628157103535?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20%E2%80%A2%20Soerya%20Sumantri%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20%E2%80%A2%20Soerya%20Sumantri%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%201%2C298%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Soerya%20Sumantri%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-soerya-sumantri%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280815-7103-535%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-soerya-sumantri.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Soerya%20Sumantri%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/628157103535?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20%E2%80%A2%20Soerya%20Sumantri%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20%E2%80%A2%20Soerya%20Sumantri%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%201%2C298%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20%E2%80%A2%20Soerya%20Sumantri%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-soerya-sumantri%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280815-7103-535%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-soerya-sumantri.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20%E2%80%A2%20Soerya%20Sumantri%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/622127517007?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AHairnerds%20Studio%20Kebayoran%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AHairnerds%20Studio%20Kebayoran%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C275%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AHairnerds%20Studio%20Kebayoran%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/hairnerds-studio-kebayoran%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28021%29%2027517007%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.hairnerds-studio-kebayora.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AHairnerds%20Studio%20Kebayoran%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2839,13 +2839,13 @@
     <t>https://wa.me/6282260659556?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AOdysen%20Barbershop%20Pondok%20Labu%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AOdysen%20Barbershop%20Pondok%20Labu%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C264%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AOdysen%20Barbershop%20Pondok%20Labu%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/odysen-barbershop-pondok-labu%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280822-6065-9556%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.odysen-barbershop-pondok-.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AOdysen%20Barbershop%20Pondok%20Labu%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6281323674385?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20%E2%80%A2%20Antapani%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20%E2%80%A2%20Antapani%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C247%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Antapani%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-antapani%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280813-2367-4385%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-antapani.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Antapani%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
-  </si>
-  <si>
-    <t>https://wa.me/6287891770824?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACHIEF%20BARBERSHOP%20-%20SABANG%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACHIEF%20BARBERSHOP%20-%20SABANG%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C240%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACHIEF%20BARBERSHOP%20-%20SABANG%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/chief-barbershop-sabang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280878-9177-0824%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.chief-barbershop-sabang.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACHIEF%20BARBERSHOP%20-%20SABANG%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
-  </si>
-  <si>
-    <t>https://wa.me/6285659339635?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2Abarberfits%20%E2%80%A2%20Pandawa%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2Abarberfits%20%E2%80%A2%20Pandawa%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%201%2C211%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2Abarberfits%20%E2%80%A2%20Pandawa%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberfits-pandawa%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280856-5933-9635%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberfits-pandawa.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2Abarberfits%20%E2%80%A2%20Pandawa%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6281323674385?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20%E2%80%A2%20Antapani%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20%E2%80%A2%20Antapani%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C247%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20%E2%80%A2%20Antapani%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-antapani%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280813-2367-4385%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-antapani.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20%E2%80%A2%20Antapani%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+  </si>
+  <si>
+    <t>https://wa.me/6287891770824?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AChief%20Barbershop%20-%20Sabang%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AChief%20Barbershop%20-%20Sabang%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C240%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AChief%20Barbershop%20-%20Sabang%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/chief-barbershop-sabang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280878-9177-0824%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.chief-barbershop-sabang.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AChief%20Barbershop%20-%20Sabang%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+  </si>
+  <si>
+    <t>https://wa.me/6285659339635?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberfits%20%E2%80%A2%20Pandawa%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberfits%20%E2%80%A2%20Pandawa%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%201%2C211%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberfits%20%E2%80%A2%20Pandawa%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberfits-pandawa%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280856-5933-9635%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberfits-pandawa.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberfits%20%E2%80%A2%20Pandawa%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6285723544694?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AKanaka%20Barbershop%20Cimahi%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AKanaka%20Barbershop%20Cimahi%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C206%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AKanaka%20Barbershop%20Cimahi%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/kanaka-barbershop-cimahi%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280857-2354-4694%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.kanaka-barbershop-cimahi.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AKanaka%20Barbershop%20Cimahi%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2854,13 +2854,13 @@
     <t>https://wa.me/6285188344170?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2APixel%20Barbershop%20Wisma%20Asri%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2APixel%20Barbershop%20Wisma%20Asri%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%201%2C199%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2APixel%20Barbershop%20Wisma%20Asri%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/pixel-barbershop-wisma-asri%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280851-8834-4170%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.pixel-barbershop-wisma-as.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2APixel%20Barbershop%20Wisma%20Asri%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6285861518608?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20%E2%80%A2%20Mekar%20Wangi%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20%E2%80%A2%20Mekar%20Wangi%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C194%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Mekar%20Wangi%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-mekar-wangi%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280858-6151-8608%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-mekar-wangi.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Mekar%20Wangi%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6285861518608?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20%E2%80%A2%20Mekar%20Wangi%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20%E2%80%A2%20Mekar%20Wangi%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C194%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20%E2%80%A2%20Mekar%20Wangi%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-mekar-wangi%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280858-6151-8608%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-mekar-wangi.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20%E2%80%A2%20Mekar%20Wangi%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281313439432?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Premiere%20Sutami%20Bandung%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Premiere%20Sutami%20Bandung%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C164%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Premiere%20Sutami%20Bandung%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-premiere-sutami-bandung%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280813-1343-9432%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-premie.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Premiere%20Sutami%20Bandung%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6287725241193?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ASUMA%20Barber%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ASUMA%20Barber%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%201%2C127%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ASUMA%20Barber%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/suma-barber%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280877-2524-1193%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.suma-barber.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ASUMA%20Barber%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6287725241193?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ASuma%20Barber%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ASuma%20Barber%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%201%2C127%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ASuma%20Barber%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/suma-barber%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280877-2524-1193%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.suma-barber.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ASuma%20Barber%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6285888088013?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AHairnerds%20Studio%20Bintaro%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AHairnerds%20Studio%20Bintaro%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%201%2C088%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AHairnerds%20Studio%20Bintaro%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/hairnerds-studio-bintaro%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280858-8808-8013%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.hairnerds-studio-bintaro.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AHairnerds%20Studio%20Bintaro%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2869,7 +2869,7 @@
     <t>https://wa.me/6285974474110?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACulture%20Barbershop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACulture%20Barbershop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%201%2C075%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACulture%20Barbershop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/culture-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280859-7447-4110%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.culture-barbershop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACulture%20Barbershop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6281519282888?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20%E2%80%A2%20Summarecon%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20%E2%80%A2%20Summarecon%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C060%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Summarecon%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-summarecon%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280815-1928-2888%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-summarecon.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Summarecon%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6281519282888?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20%E2%80%A2%20Summarecon%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20%E2%80%A2%20Summarecon%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C060%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20%E2%80%A2%20Summarecon%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-summarecon%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280815-1928-2888%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-summarecon.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20%E2%80%A2%20Summarecon%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6285811065697?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AHaircoolest%20Barbershop%20%7C%20Petojo%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AHaircoolest%20Barbershop%20%7C%20Petojo%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%201%2C028%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AHaircoolest%20Barbershop%20%7C%20Petojo%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/haircoolest-barbershop-petojo%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280858-1106-5697%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.haircoolest-barbershop-pe.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AHaircoolest%20Barbershop%20%7C%20Petojo%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2881,7 +2881,7 @@
     <t>https://wa.me/628179345934?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AChief%20Barbershop%20-%20Como%20Park%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AChief%20Barbershop%20-%20Como%20Park%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%201%2C003%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AChief%20Barbershop%20-%20Como%20Park%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/chief-barbershop-como-park%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280817-9345-934%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.chief-barbershop-como-par.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AChief%20Barbershop%20-%20Como%20Park%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/62816838055?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20%E2%80%A2%20Padjajaran%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20%E2%80%A2%20Padjajaran%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20984%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Padjajaran%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-padjajaran%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280816-838-055%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-padjajaran.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Padjajaran%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/62816838055?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20%E2%80%A2%20Padjajaran%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20%E2%80%A2%20Padjajaran%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20984%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20%E2%80%A2%20Padjajaran%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-padjajaran%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280816-838-055%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-padjajaran.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20%E2%80%A2%20Padjajaran%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6282260349485?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Buah%20Batu%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Buah%20Batu%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20968%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Buah%20Batu%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-buah-batu%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280822-6034-9485%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-buah-b.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Buah%20Batu%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2893,19 +2893,19 @@
     <t>https://wa.me/6281770003750?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AGentology%20Barbershop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AGentology%20Barbershop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20926%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AGentology%20Barbershop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/gentology-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280817-7000-3750%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.gentology-barbershop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AGentology%20Barbershop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/622172797253?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AHAIRSTUDIO%20SALON%20%26%20BARBER%20CIPETE%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AHAIRSTUDIO%20SALON%20%26%20BARBER%20CIPETE%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20870%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AHAIRSTUDIO%20SALON%20%26%20BARBER%20CIPETE%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/hairstudio-salon-barber-cipete%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28021%29%2072797253%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.hairstudio-salon-barber-c.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AHAIRSTUDIO%20SALON%20%26%20BARBER%20CIPETE%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/622172797253?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AHairstudio%20Salon%20%26%20Barber%20Cipete%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AHairstudio%20Salon%20%26%20Barber%20Cipete%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20870%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AHairstudio%20Salon%20%26%20Barber%20Cipete%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/hairstudio-salon-barber-cipete%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28021%29%2072797253%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.hairstudio-salon-barber-c.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AHairstudio%20Salon%20%26%20Barber%20Cipete%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281288838092?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ATohang%27s%20Barber%20Cawang%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ATohang%27s%20Barber%20Cawang%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20855%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ATohang%27s%20Barber%20Cawang%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/tohang-s-barber-cawang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-8883-8092%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.tohang-s-barber-cawang.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ATohang%27s%20Barber%20Cawang%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6282117213856?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABARBERLABS%20HQ%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABARBERLABS%20HQ%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%20845%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABARBERLABS%20HQ%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberlabs-hq%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-1721-3856%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberlabs-hq.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABARBERLABS%20HQ%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6282117213856?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberlabs%20Hq%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberlabs%20Hq%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%20845%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberlabs%20Hq%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberlabs-hq%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-1721-3856%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberlabs-hq.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberlabs%20Hq%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281221958355?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AUrban%20Haircut%20Studio%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AUrban%20Haircut%20Studio%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%20824%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AUrban%20Haircut%20Studio%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/urban-haircut-studio%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-2195-8355%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.urban-haircut-studio.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AUrban%20Haircut%20Studio%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/62816988055?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20%E2%80%A2%20Progo%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20%E2%80%A2%20Progo%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20797%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Progo%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-progo%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280816-988-055%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-progo.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Progo%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/62816988055?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20%E2%80%A2%20Progo%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20%E2%80%A2%20Progo%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20797%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20%E2%80%A2%20Progo%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-progo%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280816-988-055%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-progo.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20%E2%80%A2%20Progo%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/622220580000?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ATravourse%20%7C%20Garuda%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ATravourse%20%7C%20Garuda%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20791%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ATravourse%20%7C%20Garuda%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/travourse-garuda%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28022%29%2020580000%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.travourse-garuda.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ATravourse%20%7C%20Garuda%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2917,7 +2917,7 @@
     <t>https://wa.me/628561077736?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ATheboxteam%20by%20Barberbox%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ATheboxteam%20by%20Barberbox%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20790%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ATheboxteam%20by%20Barberbox%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/theboxteam-by-barberbox%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280856-1077-736%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.theboxteam-by-barberbox.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ATheboxteam%20by%20Barberbox%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/628157003535?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20%E2%80%A2%20Ramdhan%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20%E2%80%A2%20Ramdhan%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20771%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Ramdhan%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-ramdhan%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280815-7003-535%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-ramdhan.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Ramdhan%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/628157003535?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20%E2%80%A2%20Ramdhan%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20%E2%80%A2%20Ramdhan%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20771%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20%E2%80%A2%20Ramdhan%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-ramdhan%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280815-7003-535%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-ramdhan.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20%E2%80%A2%20Ramdhan%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6287822212314?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACulture%20Barbershop%20Arcamanik%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACulture%20Barbershop%20Arcamanik%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20770%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACulture%20Barbershop%20Arcamanik%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/culture-barbershop-arcamanik%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280878-2221-2314%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.culture-barbershop-arcama.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACulture%20Barbershop%20Arcamanik%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2926,19 +2926,19 @@
     <t>https://wa.me/6282338195915?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Bintaro%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Bintaro%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.5%20%E2%AD%90%20dari%20762%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Bintaro%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-bintaro%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280823-3819-5915%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-bintar.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Bintaro%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/62816618055?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20Naripan%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20Naripan%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20758%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20Naripan%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-naripan%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280816-618-055%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-naripan.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20Naripan%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/62816618055?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20Naripan%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20Naripan%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20758%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20Naripan%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-naripan%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280816-618-055%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-naripan.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20Naripan%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/628569933330?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarber%20Day%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarber%20Day%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20750%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarber%20Day%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barber-day%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280856-9933-330%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barber-day.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarber%20Day%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6282210007020?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AHAIRHAUS%20Bekasi%20-%20Barbershop%20%26%20Salon%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AHAIRHAUS%20Bekasi%20-%20Barbershop%20%26%20Salon%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20740%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AHAIRHAUS%20Bekasi%20-%20Barbershop%20%26%20Salon%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/hairhaus-bekasi-barbershop-salon%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280822-1000-7020%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.hairhaus-bekasi-barbersho.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AHAIRHAUS%20Bekasi%20-%20Barbershop%20%26%20Salon%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6282210007020?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AHairhaus%20Bekasi%20-%20Barbershop%20%26%20Salon%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AHairhaus%20Bekasi%20-%20Barbershop%20%26%20Salon%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20740%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AHairhaus%20Bekasi%20-%20Barbershop%20%26%20Salon%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/hairhaus-bekasi-barbershop-salon%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280822-1000-7020%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.hairhaus-bekasi-barbersho.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AHairhaus%20Bekasi%20-%20Barbershop%20%26%20Salon%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6282120477887?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AMoxie%20Hair%20Studio%20202%20%28Barbershop%29%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AMoxie%20Hair%20Studio%20202%20%28Barbershop%29%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20739%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AMoxie%20Hair%20Studio%20202%20%28Barbershop%29%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/moxie-hair-studio-202-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-2047-7887%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.moxie-hair-studio-202-bar.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AMoxie%20Hair%20Studio%20202%20%28Barbershop%29%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6282142011160?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACAPTAIN%20BARBERSHOP%20DUTAMAS%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACAPTAIN%20BARBERSHOP%20DUTAMAS%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.6%20%E2%AD%90%20dari%20699%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACAPTAIN%20BARBERSHOP%20DUTAMAS%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-dutamas%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-4201-1160%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-dutama.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACAPTAIN%20BARBERSHOP%20DUTAMAS%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6282142011160?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Dutamas%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Dutamas%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.6%20%E2%AD%90%20dari%20699%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Dutamas%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-dutamas%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-4201-1160%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-dutama.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Dutamas%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281286002298?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABow%20Barbershop%20Jelambar%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABow%20Barbershop%20Jelambar%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20688%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABow%20Barbershop%20Jelambar%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/bow-barbershop-jelambar%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-8600-2298%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.bow-barbershop-jelambar.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABow%20Barbershop%20Jelambar%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2950,7 +2950,7 @@
     <t>https://wa.me/6289531332958?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AMoregan%20Barbershop%20Meruya%20Ilir%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AMoregan%20Barbershop%20Meruya%20Ilir%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20685%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AMoregan%20Barbershop%20Meruya%20Ilir%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/moregan-barbershop-meruya-ilir%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280895-3133-2958%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.moregan-barbershop-meruya.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AMoregan%20Barbershop%20Meruya%20Ilir%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/62895326709996?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AAD_BARBER%20TELKOM%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AAD_BARBER%20TELKOM%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20682%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AAD_BARBER%20TELKOM%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/adbarber-telkom%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280895-3267-09996%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.adbarber-telkom.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AAD_BARBER%20TELKOM%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/62895326709996?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AAd_barber%20Telkom%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AAd_barber%20Telkom%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20682%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AAd_barber%20Telkom%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/adbarber-telkom%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280895-3267-09996%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.adbarber-telkom.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AAd_barber%20Telkom%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281332993864?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Sunda%20Bandung%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Sunda%20Bandung%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20681%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Sunda%20Bandung%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-sunda-bandung%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280813-3299-3864%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-sunda-.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Sunda%20Bandung%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2959,19 +2959,19 @@
     <t>https://wa.me/6281221186234?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ADe%20Fred%20Barber%20%26%20Shop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ADe%20Fred%20Barber%20%26%20Shop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%20678%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ADe%20Fred%20Barber%20%26%20Shop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/de-fred-barber-shop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-2118-6234%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.de-fred-barber-shop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ADe%20Fred%20Barber%20%26%20Shop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6282299942377?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20Karawang%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20Karawang%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20657%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20Karawang%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-karawang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280822-9994-2377%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-karawang.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20Karawang%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6282299942377?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20Karawang%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20Karawang%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20657%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20Karawang%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-karawang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280822-9994-2377%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-karawang.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20Karawang%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6287878672150?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ARamo%20Barbershop%20Setiabudi%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ARamo%20Barbershop%20Setiabudi%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.8%20%E2%AD%90%20dari%20656%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ARamo%20Barbershop%20Setiabudi%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/ramo-barbershop-setiabudi%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280878-7867-2150%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.ramo-barbershop-setiabudi.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ARamo%20Barbershop%20Setiabudi%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6281288991205?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberExpress%20Kemang%20Barbershop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberExpress%20Kemang%20Barbershop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20622%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberExpress%20Kemang%20Barbershop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberexpress-kemang-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-8899-1205%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberexpress-kemang-barb.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberExpress%20Kemang%20Barbershop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6281288991205?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberexpress%20Kemang%20Barbershop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberexpress%20Kemang%20Barbershop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20622%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberexpress%20Kemang%20Barbershop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberexpress-kemang-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-8899-1205%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberexpress-kemang-barb.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberexpress%20Kemang%20Barbershop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6285281306657?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Pakubuwono%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Pakubuwono%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.4%20%E2%AD%90%20dari%20622%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Pakubuwono%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-pakubuwono%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280852-8130-6657%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-pakubu.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Pakubuwono%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6281227777615?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AMASIF%20Barber%20House%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AMASIF%20Barber%20House%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20619%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AMASIF%20Barber%20House%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/masif-barber-house%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-2777-7615%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.masif-barber-house.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AMASIF%20Barber%20House%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6281227777615?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AMasif%20Barber%20House%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AMasif%20Barber%20House%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%285.0%20%E2%AD%90%20dari%20619%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AMasif%20Barber%20House%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/masif-barber-house%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-2777-7615%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.masif-barber-house.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AMasif%20Barber%20House%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6285280050209?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Tanjung%20Duren%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Tanjung%20Duren%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.6%20%E2%AD%90%20dari%20615%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Tanjung%20Duren%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-tanjung-duren%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280852-8005-0209%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-tanjun.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Tanjung%20Duren%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -2980,16 +2980,16 @@
     <t>https://wa.me/6282142011162?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Depok%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Depok%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20608%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Depok%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-depok%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280821-4201-1162%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-depok.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Depok%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/6285179785109?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ARock%20n%20Roll%20Haircutting%20%26%20Makeover%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ARock%20n%20Roll%20Haircutting%20%26%20Makeover%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.5%20%E2%AD%90%20dari%20606%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ARock%20n%20Roll%20Haircutting%20%26%20Makeover%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/rock-n-roll-haircutting-makeover%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280851-7978-5109%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.rock-n-roll-haircutting-m.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ARock%20n%20Roll%20Haircutting%20%26%20Makeover%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
-  </si>
-  <si>
-    <t>https://wa.me/6281998888167?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AMANCAVE%20BARBERSHOP%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AMANCAVE%20BARBERSHOP%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20593%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AMANCAVE%20BARBERSHOP%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/mancave-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280819-9888-8167%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.mancave-barbershop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AMANCAVE%20BARBERSHOP%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
-  </si>
-  <si>
-    <t>https://wa.me/6281803974879?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AGroomify%20Barbershop%20MONOCHROME%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AGroomify%20Barbershop%20MONOCHROME%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20590%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AGroomify%20Barbershop%20MONOCHROME%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/groomify-barbershop-monochrome%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280818-0397-4879%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.groomify-barbershop-monoc.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AGroomify%20Barbershop%20MONOCHROME%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
-  </si>
-  <si>
-    <t>https://wa.me/6282260351173?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarBerBos%20%E2%80%A2%20Maskumambang%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarBerBos%20%E2%80%A2%20Maskumambang%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20588%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Maskumambang%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-maskumambang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280822-6035-1173%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-maskumambang.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarBerBos%20%E2%80%A2%20Maskumambang%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/6285179785109?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ARock%20N%20Roll%20Haircutting%20%26%20Makeover%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ARock%20N%20Roll%20Haircutting%20%26%20Makeover%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.5%20%E2%AD%90%20dari%20606%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ARock%20N%20Roll%20Haircutting%20%26%20Makeover%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/rock-n-roll-haircutting-makeover%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280851-7978-5109%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.rock-n-roll-haircutting-m.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ARock%20N%20Roll%20Haircutting%20%26%20Makeover%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+  </si>
+  <si>
+    <t>https://wa.me/6281998888167?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AMancave%20Barbershop%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AMancave%20Barbershop%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20593%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AMancave%20Barbershop%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/mancave-barbershop%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280819-9888-8167%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.mancave-barbershop.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AMancave%20Barbershop%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+  </si>
+  <si>
+    <t>https://wa.me/6281803974879?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2AGroomify%20Barbershop%20Monochrome%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2AGroomify%20Barbershop%20Monochrome%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20590%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2AGroomify%20Barbershop%20Monochrome%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/groomify-barbershop-monochrome%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280818-0397-4879%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.groomify-barbershop-monoc.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2AGroomify%20Barbershop%20Monochrome%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+  </si>
+  <si>
+    <t>https://wa.me/6282260351173?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbos%20%E2%80%A2%20Maskumambang%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbos%20%E2%80%A2%20Maskumambang%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20588%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbos%20%E2%80%A2%20Maskumambang%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbos-maskumambang%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280822-6035-1173%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbos-maskumambang.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbos%20%E2%80%A2%20Maskumambang%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>https://wa.me/6281211105690?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ACaptain%20Barbershop%20Grogol%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ACaptain%20Barbershop%20Grogol%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.7%20%E2%AD%90%20dari%20583%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ACaptain%20Barbershop%20Grogol%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/captain-barbershop-grogol%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280812-1110-5690%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.captain-barbershop-grogol.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ACaptain%20Barbershop%20Grogol%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
@@ -3010,7 +3010,7 @@
     <t>https://wa.me/6281320234545?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ARuang%20Pangkas%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ARuang%20Pangkas%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.9%20%E2%AD%90%20dari%20555%20ulasan%20pelanggan%20di%20Bandung%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ARuang%20Pangkas%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/ruang-pangkas%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%280813-2023-4545%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.ruang-pangkas.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ARuang%20Pangkas%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
-    <t>https://wa.me/622127654089?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABARBERBAR%20Lebak%20Bulus%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABARBERBAR%20Lebak%20Bulus%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.5%20%E2%AD%90%20dari%20555%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABARBERBAR%20Lebak%20Bulus%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbar-lebak-bulus%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28021%29%2027654089%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbar-lebak-bulus.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABARBERBAR%20Lebak%20Bulus%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
+    <t>https://wa.me/622127654089?text=Halo%20Bro%20/%20Tim%20Manajemen%20%2ABarberbar%20Lebak%20Bulus%2A%2C%0A%0ASalam%20kenal%21%20Saya%20perhatikan%20%2ABarberbar%20Lebak%20Bulus%2A%20memiliki%20reputasi%20yang%20sangat%20keren%20di%20Google%20Maps%20%284.5%20%E2%AD%90%20dari%20555%20ulasan%20pelanggan%20di%20Jakarta%20Selatan%29.%0A%0AMelihat%20antusiasme%20pelanggan%20yang%20begitu%20tinggi%2C%20kami%20berinisiatif%20membuatkan%20preview%20website%20profil%20modern%20khusus%20untuk%20%2ABarberbar%20Lebak%20Bulus%2A%2C%20lengkap%20dengan%20sistem%20reservasi%20WhatsApp%20otomatis%20langsung%20ke%20nomor%20Anda%3A%0A%0A%F0%9F%91%89%20Akses%20Website%20Demo%20Barbershop%20Anda%20di%20sini%3A%0Ahttps%3A//barbershop-web-demo.vercel.app/p/barberbar-lebak-bulus%0A%0AKeunggulan%20sistem%20website%20ini%3A%0A%E2%80%A2%20Desain%20Bersih%20%26%20Elegan%3A%20Tampilan%20terang%20modern%20%28Apple%20%26%20Scandinavian%20style%29%2C%20sangat%20nyaman%20dibuka%20di%20smartphone%0A%E2%80%A2%20Booking%20WhatsApp%20Otomatis%3A%20Calon%20pelanggan%20bisa%20pilih%20capster%2C%20jam%2C%20dan%20layanan%E2%80%94langsung%20masuk%20ke%20WA%20Anda%20%28%28021%29%2027654089%29%0A%E2%80%A2%20Menu%20Layanan%20%26%20Harga%20Transparan%3A%20Menampilkan%20signature%20cut%2C%20shave%2C%20dan%20creambath%0A%E2%80%A2%20Hairstyle%20Lookbook%20%26%20Face-Shape%20Guide%3A%20Edukasi%20gaya%20rambut%20untuk%20pelanggan%20Anda%0A%E2%80%A2%20Siap%20Dihubungkan%20ke%20Domain%20Resmi%20%28contoh%3A%20www.barberbar-lebak-bulus.com%29%0A%0AWebsite%20ini%20sudah%20siap%20pakai%20dan%20siap%20kami%20serahkan.%20Jika%20Anda%20atau%20tim%20manajemen%20tertarik%20untuk%20mengaktifkannya%2C%20bisa%20langsung%20hubungi%20WhatsApp%20saya%20di%20%2B62%20857-1820-3535%20atau%20klik%20tombol%20%27Klaim%20Website%20Ini%27%20di%20halaman%20demo.%0A%0ATerima%20kasih%20banyak%20bro%2C%20sukses%20terus%20untuk%20%2ABarberbar%20Lebak%20Bulus%2A%21%20%F0%9F%99%8F%E2%9C%82%EF%B8%8F</t>
   </si>
   <si>
     <t>Jl. Terusan Batik Halus No.17, Sukaluyu, Kec. Cibeunying Kaler, Kota Bandung, Jawa Barat 40123</t>

</xml_diff>